<commit_message>
i18n: fully localize the app to English
Translate all in-code text to English: comments, docstrings, CLI menu/
messages, log output, error messages, and the generated-text templates
(Slack/Teams/email tones, X/LinkedIn/Qiita posts). Also translate setup
scripts, config comments, and sample data. Switch Windows clipboard
encoding from cp932 to utf-16-le for proper Unicode support.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/sample_sales.xlsx
+++ b/samples/sample_sales.xlsx
@@ -419,29 +419,29 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>売上高</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>前年売上</t>
+          <t>PrevYear</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>利益</t>
+          <t>Profit</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4月</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -457,7 +457,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5月</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -473,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6月</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -489,7 +489,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7月</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>8月</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -521,7 +521,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9月</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="B7" t="n">

</xml_diff>